<commit_message>
update train.py batch size 16
</commit_message>
<xml_diff>
--- a/Test3_vggnet/Record.xlsx
+++ b/Test3_vggnet/Record.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renhonglow/Library/Mobile Documents/com~apple~CloudDocs/School/yjs/Learn/DL/Test3_vggnet/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renhonglow/Desktop/DL/Test3_vggnet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C038CB-22EE-6643-B867-74D292E1E0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007E392D-5235-F244-A4E7-D86A5FE66074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2700" yWindow="680" windowWidth="26660" windowHeight="17380" xr2:uid="{FEBCBEC6-E82C-7B45-A035-B8783A5A7100}"/>
+    <workbookView xWindow="-30500" yWindow="-640" windowWidth="24980" windowHeight="17380" xr2:uid="{FEBCBEC6-E82C-7B45-A035-B8783A5A7100}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -105,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -116,6 +116,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -484,9 +487,9 @@
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
       <c r="K2" s="2">
         <v>0.3</v>
       </c>
@@ -503,28 +506,19 @@
         <v>4</v>
       </c>
       <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
         <v>16</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>32</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>64</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>128</v>
-      </c>
-      <c r="F3">
-        <v>64</v>
-      </c>
-      <c r="G3">
-        <v>32</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>16</v>
       </c>
       <c r="J3">
         <v>256</v>
@@ -552,30 +546,13 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>10</v>
-      </c>
-      <c r="C4">
-        <v>30</v>
-      </c>
-      <c r="D4">
-        <v>50</v>
-      </c>
-      <c r="E4">
+      <c r="B4" s="2">
         <v>100</v>
       </c>
-      <c r="F4">
-        <v>100</v>
-      </c>
-      <c r="G4">
-        <v>100</v>
-      </c>
-      <c r="H4">
-        <v>100</v>
-      </c>
-      <c r="I4">
-        <v>100</v>
-      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
       <c r="J4">
         <v>100</v>
       </c>
@@ -602,30 +579,13 @@
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="2">
         <v>1E-4</v>
       </c>
-      <c r="C5">
-        <v>1E-3</v>
-      </c>
-      <c r="D5">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="E5">
-        <v>1E-4</v>
-      </c>
-      <c r="F5">
-        <v>1E-4</v>
-      </c>
-      <c r="G5">
-        <v>1E-4</v>
-      </c>
-      <c r="H5">
-        <v>1E-4</v>
-      </c>
-      <c r="I5">
-        <v>1E-4</v>
-      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
       <c r="J5">
         <v>1E-4</v>
       </c>
@@ -656,22 +616,16 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>1.1519999999999999</v>
-      </c>
-      <c r="C7">
-        <v>1.601</v>
+        <v>0.313</v>
+      </c>
+      <c r="D7">
+        <v>0.28399999999999997</v>
       </c>
       <c r="E7">
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="F7">
         <v>0.28299999999999997</v>
-      </c>
-      <c r="F7">
-        <v>0.26800000000000002</v>
-      </c>
-      <c r="G7">
-        <v>0.28399999999999997</v>
-      </c>
-      <c r="H7">
-        <v>0.313</v>
       </c>
       <c r="J7">
         <v>0.33300000000000002</v>
@@ -682,22 +636,16 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.54400000000000004</v>
-      </c>
-      <c r="C8">
-        <v>0.245</v>
+        <v>0.81899999999999995</v>
+      </c>
+      <c r="D8">
+        <v>0.82699999999999996</v>
       </c>
       <c r="E8">
+        <v>0.81599999999999995</v>
+      </c>
+      <c r="F8">
         <v>0.79100000000000004</v>
-      </c>
-      <c r="F8">
-        <v>0.81599999999999995</v>
-      </c>
-      <c r="G8">
-        <v>0.82699999999999996</v>
-      </c>
-      <c r="H8">
-        <v>0.81899999999999995</v>
       </c>
       <c r="J8">
         <v>0.79400000000000004</v>
@@ -849,7 +797,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="B1:J1"/>
@@ -857,7 +805,9 @@
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="H14:J14"/>
-    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
batch size 32 to 64
</commit_message>
<xml_diff>
--- a/Test3_vggnet/Record.xlsx
+++ b/Test3_vggnet/Record.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renhonglow/Desktop/DL/Test3_vggnet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA2E2618-E7BB-B249-8F84-AAB0C8A168F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14801239-2B1E-4F42-8B8D-F30F75F75FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29300" yWindow="-800" windowWidth="24980" windowHeight="17380" xr2:uid="{FEBCBEC6-E82C-7B45-A035-B8783A5A7100}"/>
+    <workbookView xWindow="-26680" yWindow="-1860" windowWidth="24980" windowHeight="17380" xr2:uid="{FEBCBEC6-E82C-7B45-A035-B8783A5A7100}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
   <si>
     <t>Vgg16</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>Val Accurancy</t>
+  </si>
+  <si>
+    <t>safari</t>
   </si>
 </sst>
 </file>
@@ -520,11 +523,14 @@
       <c r="F3">
         <v>128</v>
       </c>
+      <c r="I3">
+        <v>256</v>
+      </c>
       <c r="J3">
-        <v>256</v>
+        <v>16</v>
       </c>
       <c r="K3">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L3">
         <v>32</v>
@@ -553,6 +559,9 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
+      <c r="I4">
+        <v>100</v>
+      </c>
       <c r="J4">
         <v>100</v>
       </c>
@@ -586,6 +595,9 @@
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
+      <c r="I5">
+        <v>1E-4</v>
+      </c>
       <c r="J5">
         <v>1E-4</v>
       </c>
@@ -630,11 +642,17 @@
       <c r="F7">
         <v>0.28299999999999997</v>
       </c>
+      <c r="I7">
+        <v>0.33300000000000002</v>
+      </c>
       <c r="J7">
-        <v>0.33300000000000002</v>
-      </c>
-      <c r="K7">
         <v>0.27800000000000002</v>
+      </c>
+      <c r="K7" t="s">
+        <v>9</v>
+      </c>
+      <c r="L7">
+        <v>0.378</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -656,11 +674,14 @@
       <c r="F8">
         <v>0.79100000000000004</v>
       </c>
+      <c r="I8">
+        <v>0.79400000000000004</v>
+      </c>
       <c r="J8">
-        <v>0.79400000000000004</v>
-      </c>
-      <c r="K8">
         <v>0.83799999999999997</v>
+      </c>
+      <c r="L8">
+        <v>0.79700000000000004</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
bs 8 2 64
</commit_message>
<xml_diff>
--- a/Test3_vggnet/Record.xlsx
+++ b/Test3_vggnet/Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renhonglow/Desktop/DL/Test3_vggnet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14801239-2B1E-4F42-8B8D-F30F75F75FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C9350C-3FF7-6649-B883-4292113B8288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-26680" yWindow="-1860" windowWidth="24980" windowHeight="17380" xr2:uid="{FEBCBEC6-E82C-7B45-A035-B8783A5A7100}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="9">
   <si>
     <t>Vgg16</t>
   </si>
@@ -64,9 +64,6 @@
   <si>
     <t>Val Accurancy</t>
   </si>
-  <si>
-    <t>safari</t>
-  </si>
 </sst>
 </file>
 
@@ -88,12 +85,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -108,12 +111,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -467,42 +471,42 @@
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="6">
         <v>0.1</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="K2" s="3">
+      <c r="K2" s="4">
         <v>0.3</v>
       </c>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3">
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4">
         <v>0.5</v>
       </c>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -552,13 +556,13 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
         <v>100</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
       <c r="I4">
         <v>100</v>
       </c>
@@ -588,13 +592,13 @@
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3">
-        <v>1E-4</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="B5" s="4">
+        <v>1E-4</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
       <c r="I5">
         <v>1E-4</v>
       </c>
@@ -648,8 +652,8 @@
       <c r="J7">
         <v>0.27800000000000002</v>
       </c>
-      <c r="K7" t="s">
-        <v>9</v>
+      <c r="K7" s="3">
+        <v>1.6</v>
       </c>
       <c r="L7">
         <v>0.378</v>
@@ -680,6 +684,9 @@
       <c r="J8">
         <v>0.83799999999999997</v>
       </c>
+      <c r="K8" s="3">
+        <v>0.245</v>
+      </c>
       <c r="L8">
         <v>0.79700000000000004</v>
       </c>
@@ -688,37 +695,37 @@
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="4">
         <v>0.1</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3">
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4">
         <v>0.3</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3">
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4">
         <v>0.5</v>
       </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
@@ -772,7 +779,7 @@
         <v>30</v>
       </c>
       <c r="G16">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H16">
         <v>10</v>
@@ -804,7 +811,7 @@
         <v>1E-3</v>
       </c>
       <c r="G17">
-        <v>5.0000000000000001E-3</v>
+        <v>1E-4</v>
       </c>
       <c r="H17">
         <v>1E-4</v>
@@ -818,10 +825,16 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
+      <c r="G18">
+        <v>0.34100000000000003</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="G19">
+        <v>0.79400000000000004</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>